<commit_message>
data: update blank rows
</commit_message>
<xml_diff>
--- a/pronouns_game/db_pronouns_social-adressing_v1.xlsx
+++ b/pronouns_game/db_pronouns_social-adressing_v1.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="329" uniqueCount="106">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="351" uniqueCount="107">
   <si>
     <t>adressing relation</t>
   </si>
@@ -82,6 +82,9 @@
     <t xml:space="preserve">sahbi </t>
   </si>
   <si>
+    <t>-</t>
+  </si>
+  <si>
     <t>Nepal</t>
   </si>
   <si>
@@ -103,13 +106,19 @@
     <t>Urdu</t>
   </si>
   <si>
-    <t>تم (tum) / آپ (aap)</t>
+    <t>تم (tum)</t>
   </si>
   <si>
     <t>میں</t>
   </si>
   <si>
-    <t>tum / تم = casual among friends; aap / آپ = more polite</t>
+    <t>tum / تم = casual among friends</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> آپ (aap)</t>
+  </si>
+  <si>
+    <t>aap / آپ = more polite</t>
   </si>
   <si>
     <t>Vietnam</t>
@@ -145,7 +154,7 @@
     <t>informal</t>
   </si>
   <si>
-    <t>younger person (~younger sibling's generation)</t>
+    <t>younger person (~same generation)</t>
   </si>
   <si>
     <t>Mandarin</t>
@@ -175,13 +184,7 @@
     <t>细妹 (sè-muē)</t>
   </si>
   <si>
-    <t>-</t>
-  </si>
-  <si>
     <t>तँ (ta)</t>
-  </si>
-  <si>
-    <t>urdu</t>
   </si>
   <si>
     <t>تم (tum) or تو (tu)</t>
@@ -205,7 +208,7 @@
     <t>i/me as female speaker</t>
   </si>
   <si>
-    <t>older person (~older sibling's generation)</t>
+    <t>older person (~same generation)</t>
   </si>
   <si>
     <t>哥哥 (gēge)</t>
@@ -229,13 +232,19 @@
     <t>तपाईं (tapai) and हजुर (Hajur)</t>
   </si>
   <si>
-    <t>بھائی (bhai / bhaiya)  or  باجی (baji / apa)</t>
+    <t xml:space="preserve">بھائی (bhai / bhaiya) </t>
   </si>
   <si>
-    <t>common to call slightly older people "bhai" (male) or "baji/apa" (female) for respect</t>
+    <t>common to call slightly older people "bhai" (male) for respect</t>
   </si>
   <si>
-    <t>middle-age person (~uncle/auntie)</t>
+    <t xml:space="preserve">  باجی (baji / apa)</t>
+  </si>
+  <si>
+    <t>common to call slightly older people "baji/apa" (female) for respect</t>
+  </si>
+  <si>
+    <t>middle-age person (~parents' gen)</t>
   </si>
   <si>
     <t>叔叔 (shūshu)</t>
@@ -271,16 +280,10 @@
     <t>aunty</t>
   </si>
   <si>
-    <t>Uncle / Aunty or چچا (chacha) / خالہ (khala)</t>
+    <t>Uncle / چچا (chacha)</t>
   </si>
   <si>
-    <t>"Uncle" &amp; "Auntie" (English words) are very commonly used even when speaking Urdu</t>
-  </si>
-  <si>
-    <t>Singapore</t>
-  </si>
-  <si>
-    <t>auntie</t>
+    <t>Aunty /خالہ (khala)</t>
   </si>
   <si>
     <t>chú/cậu</t>
@@ -794,10 +797,10 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:Z1032"/>
+  <dimension ref="A1:Z1033"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="18" width="35.86214285714286" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="18" width="47.14785714285715" customWidth="1" bestFit="1"/>
     <col min="2" max="2" style="18" width="29.290714285714284" customWidth="1" bestFit="1"/>
     <col min="3" max="3" style="18" width="13.576428571428572" customWidth="1" bestFit="1"/>
     <col min="4" max="4" style="19" width="33.14785714285715" customWidth="1" bestFit="1"/>
@@ -992,7 +995,9 @@
       <c r="D5" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="E5" s="3"/>
+      <c r="E5" s="3" t="s">
+        <v>22</v>
+      </c>
       <c r="F5" s="3"/>
       <c r="G5" s="4"/>
       <c r="H5" s="4"/>
@@ -1020,19 +1025,19 @@
         <v>6</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G6" s="6"/>
       <c r="H6" s="6"/>
@@ -1060,59 +1065,59 @@
         <v>6</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="G7" s="4"/>
-      <c r="H7" s="4"/>
-      <c r="I7" s="4"/>
-      <c r="J7" s="4"/>
-      <c r="K7" s="4"/>
-      <c r="L7" s="4"/>
-      <c r="M7" s="4"/>
-      <c r="N7" s="4"/>
-      <c r="O7" s="4"/>
-      <c r="P7" s="4"/>
-      <c r="Q7" s="4"/>
-      <c r="R7" s="4"/>
-      <c r="S7" s="4"/>
-      <c r="T7" s="4"/>
-      <c r="U7" s="4"/>
-      <c r="V7" s="4"/>
-      <c r="W7" s="4"/>
-      <c r="X7" s="4"/>
-      <c r="Y7" s="4"/>
-      <c r="Z7" s="4"/>
+        <v>32</v>
+      </c>
+      <c r="G7" s="6"/>
+      <c r="H7" s="6"/>
+      <c r="I7" s="6"/>
+      <c r="J7" s="6"/>
+      <c r="K7" s="6"/>
+      <c r="L7" s="6"/>
+      <c r="M7" s="6"/>
+      <c r="N7" s="6"/>
+      <c r="O7" s="6"/>
+      <c r="P7" s="6"/>
+      <c r="Q7" s="6"/>
+      <c r="R7" s="6"/>
+      <c r="S7" s="6"/>
+      <c r="T7" s="6"/>
+      <c r="U7" s="6"/>
+      <c r="V7" s="6"/>
+      <c r="W7" s="6"/>
+      <c r="X7" s="6"/>
+      <c r="Y7" s="6"/>
+      <c r="Z7" s="6"/>
     </row>
     <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="18.75">
       <c r="A8" s="3" t="s">
         <v>6</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="C8" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D8" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="D8" s="3" t="s">
+      <c r="E8" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="F8" s="3" t="s">
         <v>34</v>
-      </c>
-      <c r="E8" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="F8" s="3" t="s">
-        <v>36</v>
       </c>
       <c r="G8" s="4"/>
       <c r="H8" s="4"/>
@@ -1140,19 +1145,19 @@
         <v>6</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="G9" s="4"/>
       <c r="H9" s="4"/>
@@ -1180,16 +1185,16 @@
         <v>6</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="F10" s="3" t="s">
         <v>39</v>
@@ -1220,13 +1225,13 @@
         <v>6</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="E11" s="3" t="s">
         <v>41</v>
@@ -1255,63 +1260,63 @@
       <c r="Y11" s="4"/>
       <c r="Z11" s="4"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="28.5">
-      <c r="A12" s="7" t="s">
+    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="18.75">
+      <c r="A12" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="D12" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="B12" s="7" t="s">
+      <c r="E12" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="F12" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="G12" s="4"/>
+      <c r="H12" s="4"/>
+      <c r="I12" s="4"/>
+      <c r="J12" s="4"/>
+      <c r="K12" s="4"/>
+      <c r="L12" s="4"/>
+      <c r="M12" s="4"/>
+      <c r="N12" s="4"/>
+      <c r="O12" s="4"/>
+      <c r="P12" s="4"/>
+      <c r="Q12" s="4"/>
+      <c r="R12" s="4"/>
+      <c r="S12" s="4"/>
+      <c r="T12" s="4"/>
+      <c r="U12" s="4"/>
+      <c r="V12" s="4"/>
+      <c r="W12" s="4"/>
+      <c r="X12" s="4"/>
+      <c r="Y12" s="4"/>
+      <c r="Z12" s="4"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="18.75">
+      <c r="A13" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="B13" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="C12" s="7" t="s">
-        <v>44</v>
-      </c>
-      <c r="D12" s="7" t="s">
-        <v>45</v>
-      </c>
-      <c r="E12" s="7" t="s">
-        <v>46</v>
-      </c>
-      <c r="F12" s="7"/>
-      <c r="G12" s="8"/>
-      <c r="H12" s="8"/>
-      <c r="I12" s="8"/>
-      <c r="J12" s="8"/>
-      <c r="K12" s="8"/>
-      <c r="L12" s="8"/>
-      <c r="M12" s="8"/>
-      <c r="N12" s="8"/>
-      <c r="O12" s="8"/>
-      <c r="P12" s="8"/>
-      <c r="Q12" s="8"/>
-      <c r="R12" s="8"/>
-      <c r="S12" s="8"/>
-      <c r="T12" s="8"/>
-      <c r="U12" s="8"/>
-      <c r="V12" s="8"/>
-      <c r="W12" s="8"/>
-      <c r="X12" s="8"/>
-      <c r="Y12" s="8"/>
-      <c r="Z12" s="8"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="28.5">
-      <c r="A13" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="B13" s="7" t="s">
-        <v>11</v>
-      </c>
       <c r="C13" s="7" t="s">
-        <v>12</v>
+        <v>47</v>
       </c>
       <c r="D13" s="7" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="E13" s="7" t="s">
-        <v>14</v>
-      </c>
-      <c r="F13" s="7" t="s">
-        <v>48</v>
-      </c>
+        <v>49</v>
+      </c>
+      <c r="F13" s="7"/>
       <c r="G13" s="8"/>
       <c r="H13" s="8"/>
       <c r="I13" s="8"/>
@@ -1333,9 +1338,9 @@
       <c r="Y13" s="8"/>
       <c r="Z13" s="8"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="28.5">
+    <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="18.75">
       <c r="A14" s="7" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="B14" s="7" t="s">
         <v>11</v>
@@ -1344,13 +1349,13 @@
         <v>12</v>
       </c>
       <c r="D14" s="7" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E14" s="7" t="s">
         <v>14</v>
       </c>
       <c r="F14" s="7" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="G14" s="8"/>
       <c r="H14" s="8"/>
@@ -1373,24 +1378,24 @@
       <c r="Y14" s="8"/>
       <c r="Z14" s="8"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="28.5">
+    <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="18.75">
       <c r="A15" s="7" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="D15" s="7" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="E15" s="7" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="F15" s="7" t="s">
-        <v>48</v>
+        <v>53</v>
       </c>
       <c r="G15" s="8"/>
       <c r="H15" s="8"/>
@@ -1413,9 +1418,9 @@
       <c r="Y15" s="8"/>
       <c r="Z15" s="8"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="28.5">
+    <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="18.75">
       <c r="A16" s="7" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="B16" s="7" t="s">
         <v>15</v>
@@ -1424,13 +1429,13 @@
         <v>16</v>
       </c>
       <c r="D16" s="7" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="E16" s="7" t="s">
         <v>18</v>
       </c>
       <c r="F16" s="7" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="G16" s="8"/>
       <c r="H16" s="8"/>
@@ -1453,21 +1458,25 @@
       <c r="Y16" s="8"/>
       <c r="Z16" s="8"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="28.5">
+    <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="18.75">
       <c r="A17" s="7" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="C17" s="7" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="D17" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="E17" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="F17" s="7" t="s">
         <v>53</v>
       </c>
-      <c r="E17" s="7"/>
-      <c r="F17" s="7"/>
       <c r="G17" s="8"/>
       <c r="H17" s="8"/>
       <c r="I17" s="8"/>
@@ -1489,104 +1498,102 @@
       <c r="Y17" s="8"/>
       <c r="Z17" s="8"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="28.5">
-      <c r="A18" s="9" t="s">
-        <v>43</v>
-      </c>
-      <c r="B18" s="9" t="s">
+    <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="18.75">
+      <c r="A18" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="B18" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="C18" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="D18" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="C18" s="9" t="s">
-        <v>23</v>
-      </c>
-      <c r="D18" s="9" t="s">
-        <v>54</v>
-      </c>
-      <c r="E18" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="F18" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="G18" s="10"/>
-      <c r="H18" s="10"/>
-      <c r="I18" s="10"/>
-      <c r="J18" s="10"/>
-      <c r="K18" s="10"/>
-      <c r="L18" s="10"/>
-      <c r="M18" s="10"/>
-      <c r="N18" s="10"/>
-      <c r="O18" s="10"/>
-      <c r="P18" s="10"/>
-      <c r="Q18" s="10"/>
-      <c r="R18" s="10"/>
-      <c r="S18" s="10"/>
-      <c r="T18" s="10"/>
-      <c r="U18" s="10"/>
-      <c r="V18" s="10"/>
-      <c r="W18" s="10"/>
-      <c r="X18" s="10"/>
-      <c r="Y18" s="10"/>
-      <c r="Z18" s="10"/>
+      <c r="E18" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="F18" s="7"/>
+      <c r="G18" s="8"/>
+      <c r="H18" s="8"/>
+      <c r="I18" s="8"/>
+      <c r="J18" s="8"/>
+      <c r="K18" s="8"/>
+      <c r="L18" s="8"/>
+      <c r="M18" s="8"/>
+      <c r="N18" s="8"/>
+      <c r="O18" s="8"/>
+      <c r="P18" s="8"/>
+      <c r="Q18" s="8"/>
+      <c r="R18" s="8"/>
+      <c r="S18" s="8"/>
+      <c r="T18" s="8"/>
+      <c r="U18" s="8"/>
+      <c r="V18" s="8"/>
+      <c r="W18" s="8"/>
+      <c r="X18" s="8"/>
+      <c r="Y18" s="8"/>
+      <c r="Z18" s="8"/>
     </row>
     <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="18.75">
       <c r="A19" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="B19" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="B19" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="C19" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="D19" s="9" t="s">
+        <v>56</v>
+      </c>
+      <c r="E19" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="F19" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="C19" s="7" t="s">
-        <v>55</v>
-      </c>
-      <c r="D19" s="7" t="s">
-        <v>56</v>
-      </c>
-      <c r="E19" s="7" t="s">
-        <v>30</v>
-      </c>
-      <c r="F19" s="7" t="s">
-        <v>57</v>
-      </c>
-      <c r="G19" s="8"/>
-      <c r="H19" s="8"/>
-      <c r="I19" s="8"/>
-      <c r="J19" s="8"/>
-      <c r="K19" s="8"/>
-      <c r="L19" s="8"/>
-      <c r="M19" s="8"/>
-      <c r="N19" s="8"/>
-      <c r="O19" s="8"/>
-      <c r="P19" s="8"/>
-      <c r="Q19" s="8"/>
-      <c r="R19" s="8"/>
-      <c r="S19" s="8"/>
-      <c r="T19" s="8"/>
-      <c r="U19" s="8"/>
-      <c r="V19" s="8"/>
-      <c r="W19" s="8"/>
-      <c r="X19" s="8"/>
-      <c r="Y19" s="8"/>
-      <c r="Z19" s="8"/>
+      <c r="G19" s="10"/>
+      <c r="H19" s="10"/>
+      <c r="I19" s="10"/>
+      <c r="J19" s="10"/>
+      <c r="K19" s="10"/>
+      <c r="L19" s="10"/>
+      <c r="M19" s="10"/>
+      <c r="N19" s="10"/>
+      <c r="O19" s="10"/>
+      <c r="P19" s="10"/>
+      <c r="Q19" s="10"/>
+      <c r="R19" s="10"/>
+      <c r="S19" s="10"/>
+      <c r="T19" s="10"/>
+      <c r="U19" s="10"/>
+      <c r="V19" s="10"/>
+      <c r="W19" s="10"/>
+      <c r="X19" s="10"/>
+      <c r="Y19" s="10"/>
+      <c r="Z19" s="10"/>
     </row>
     <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="18.75">
       <c r="A20" s="7" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="B20" s="7" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="C20" s="7" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="D20" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="E20" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="F20" s="7" t="s">
         <v>58</v>
-      </c>
-      <c r="E20" s="7" t="s">
-        <v>59</v>
-      </c>
-      <c r="F20" s="7" t="s">
-        <v>60</v>
       </c>
       <c r="G20" s="8"/>
       <c r="H20" s="8"/>
@@ -1611,22 +1618,22 @@
     </row>
     <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="18.75">
       <c r="A21" s="7" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="B21" s="7" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C21" s="7" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="D21" s="7" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="E21" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="F21" s="7" t="s">
         <v>61</v>
-      </c>
-      <c r="F21" s="7" t="s">
-        <v>62</v>
       </c>
       <c r="G21" s="8"/>
       <c r="H21" s="8"/>
@@ -1650,54 +1657,54 @@
       <c r="Z21" s="8"/>
     </row>
     <row x14ac:dyDescent="0.25" r="22" customHeight="1" ht="18.75">
-      <c r="A22" s="11" t="s">
+      <c r="A22" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="B22" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="C22" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="D22" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="E22" s="7" t="s">
+        <v>62</v>
+      </c>
+      <c r="F22" s="7" t="s">
         <v>63</v>
       </c>
-      <c r="B22" s="11" t="s">
-        <v>7</v>
-      </c>
-      <c r="C22" s="11" t="s">
-        <v>44</v>
-      </c>
-      <c r="D22" s="11" t="s">
-        <v>64</v>
-      </c>
-      <c r="E22" s="11" t="s">
-        <v>10</v>
-      </c>
-      <c r="F22" s="11" t="s">
-        <v>48</v>
-      </c>
-      <c r="G22" s="12"/>
-      <c r="H22" s="12"/>
-      <c r="I22" s="12"/>
-      <c r="J22" s="12"/>
-      <c r="K22" s="12"/>
-      <c r="L22" s="12"/>
-      <c r="M22" s="12"/>
-      <c r="N22" s="12"/>
-      <c r="O22" s="12"/>
-      <c r="P22" s="12"/>
-      <c r="Q22" s="12"/>
-      <c r="R22" s="12"/>
-      <c r="S22" s="12"/>
-      <c r="T22" s="12"/>
-      <c r="U22" s="12"/>
-      <c r="V22" s="12"/>
-      <c r="W22" s="12"/>
-      <c r="X22" s="12"/>
-      <c r="Y22" s="12"/>
-      <c r="Z22" s="12"/>
+      <c r="G22" s="8"/>
+      <c r="H22" s="8"/>
+      <c r="I22" s="8"/>
+      <c r="J22" s="8"/>
+      <c r="K22" s="8"/>
+      <c r="L22" s="8"/>
+      <c r="M22" s="8"/>
+      <c r="N22" s="8"/>
+      <c r="O22" s="8"/>
+      <c r="P22" s="8"/>
+      <c r="Q22" s="8"/>
+      <c r="R22" s="8"/>
+      <c r="S22" s="8"/>
+      <c r="T22" s="8"/>
+      <c r="U22" s="8"/>
+      <c r="V22" s="8"/>
+      <c r="W22" s="8"/>
+      <c r="X22" s="8"/>
+      <c r="Y22" s="8"/>
+      <c r="Z22" s="8"/>
     </row>
     <row x14ac:dyDescent="0.25" r="23" customHeight="1" ht="18.75">
       <c r="A23" s="11" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B23" s="11" t="s">
         <v>7</v>
       </c>
       <c r="C23" s="11" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="D23" s="11" t="s">
         <v>65</v>
@@ -1706,7 +1713,7 @@
         <v>10</v>
       </c>
       <c r="F23" s="11" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="G23" s="12"/>
       <c r="H23" s="12"/>
@@ -1731,22 +1738,22 @@
     </row>
     <row x14ac:dyDescent="0.25" r="24" customHeight="1" ht="18.75">
       <c r="A24" s="11" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B24" s="11" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="C24" s="11" t="s">
-        <v>12</v>
+        <v>47</v>
       </c>
       <c r="D24" s="11" t="s">
         <v>66</v>
       </c>
       <c r="E24" s="11" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="F24" s="11" t="s">
-        <v>48</v>
+        <v>53</v>
       </c>
       <c r="G24" s="12"/>
       <c r="H24" s="12"/>
@@ -1771,7 +1778,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="25" customHeight="1" ht="18.75">
       <c r="A25" s="11" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B25" s="11" t="s">
         <v>11</v>
@@ -1786,7 +1793,7 @@
         <v>14</v>
       </c>
       <c r="F25" s="11" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="G25" s="12"/>
       <c r="H25" s="12"/>
@@ -1811,22 +1818,22 @@
     </row>
     <row x14ac:dyDescent="0.25" r="26" customHeight="1" ht="18.75">
       <c r="A26" s="11" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B26" s="11" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="C26" s="11" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="D26" s="11" t="s">
         <v>68</v>
       </c>
       <c r="E26" s="11" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="F26" s="11" t="s">
-        <v>48</v>
+        <v>53</v>
       </c>
       <c r="G26" s="12"/>
       <c r="H26" s="12"/>
@@ -1851,7 +1858,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="27" customHeight="1" ht="18.75">
       <c r="A27" s="11" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B27" s="11" t="s">
         <v>15</v>
@@ -1866,7 +1873,7 @@
         <v>18</v>
       </c>
       <c r="F27" s="11" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="G27" s="12"/>
       <c r="H27" s="12"/>
@@ -1891,17 +1898,23 @@
     </row>
     <row x14ac:dyDescent="0.25" r="28" customHeight="1" ht="18.75">
       <c r="A28" s="11" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B28" s="11" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="C28" s="11" t="s">
-        <v>20</v>
-      </c>
-      <c r="D28" s="11"/>
-      <c r="E28" s="11"/>
-      <c r="F28" s="11"/>
+        <v>16</v>
+      </c>
+      <c r="D28" s="11" t="s">
+        <v>70</v>
+      </c>
+      <c r="E28" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="F28" s="11" t="s">
+        <v>53</v>
+      </c>
       <c r="G28" s="12"/>
       <c r="H28" s="12"/>
       <c r="I28" s="12"/>
@@ -1924,141 +1937,141 @@
       <c r="Z28" s="12"/>
     </row>
     <row x14ac:dyDescent="0.25" r="29" customHeight="1" ht="18.75">
-      <c r="A29" s="9" t="s">
-        <v>63</v>
-      </c>
-      <c r="B29" s="9" t="s">
+      <c r="A29" s="11" t="s">
+        <v>64</v>
+      </c>
+      <c r="B29" s="11" t="s">
+        <v>19</v>
+      </c>
+      <c r="C29" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="D29" s="11" t="s">
         <v>22</v>
       </c>
-      <c r="C29" s="9"/>
-      <c r="D29" s="9" t="s">
-        <v>70</v>
-      </c>
-      <c r="E29" s="10" t="s">
-        <v>25</v>
-      </c>
-      <c r="F29" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="G29" s="10"/>
-      <c r="H29" s="10"/>
-      <c r="I29" s="10"/>
-      <c r="J29" s="10"/>
-      <c r="K29" s="10"/>
-      <c r="L29" s="10"/>
-      <c r="M29" s="10"/>
-      <c r="N29" s="10"/>
-      <c r="O29" s="10"/>
-      <c r="P29" s="10"/>
-      <c r="Q29" s="10"/>
-      <c r="R29" s="10"/>
-      <c r="S29" s="10"/>
-      <c r="T29" s="10"/>
-      <c r="U29" s="10"/>
-      <c r="V29" s="10"/>
-      <c r="W29" s="10"/>
-      <c r="X29" s="10"/>
-      <c r="Y29" s="10"/>
-      <c r="Z29" s="10"/>
+      <c r="E29" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="F29" s="11"/>
+      <c r="G29" s="12"/>
+      <c r="H29" s="12"/>
+      <c r="I29" s="12"/>
+      <c r="J29" s="12"/>
+      <c r="K29" s="12"/>
+      <c r="L29" s="12"/>
+      <c r="M29" s="12"/>
+      <c r="N29" s="12"/>
+      <c r="O29" s="12"/>
+      <c r="P29" s="12"/>
+      <c r="Q29" s="12"/>
+      <c r="R29" s="12"/>
+      <c r="S29" s="12"/>
+      <c r="T29" s="12"/>
+      <c r="U29" s="12"/>
+      <c r="V29" s="12"/>
+      <c r="W29" s="12"/>
+      <c r="X29" s="12"/>
+      <c r="Y29" s="12"/>
+      <c r="Z29" s="12"/>
     </row>
     <row x14ac:dyDescent="0.25" r="30" customHeight="1" ht="18.75">
       <c r="A30" s="11" t="s">
-        <v>63</v>
-      </c>
-      <c r="B30" s="11" t="s">
+        <v>64</v>
+      </c>
+      <c r="B30" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="C30" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="D30" s="9" t="s">
+        <v>71</v>
+      </c>
+      <c r="E30" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="F30" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="C30" s="11" t="s">
-        <v>55</v>
-      </c>
-      <c r="D30" s="11" t="s">
-        <v>71</v>
-      </c>
-      <c r="E30" s="11" t="s">
-        <v>30</v>
-      </c>
-      <c r="F30" s="11" t="s">
-        <v>72</v>
-      </c>
-      <c r="G30" s="12"/>
-      <c r="H30" s="12"/>
-      <c r="I30" s="12"/>
-      <c r="J30" s="12"/>
-      <c r="K30" s="12"/>
-      <c r="L30" s="12"/>
-      <c r="M30" s="12"/>
-      <c r="N30" s="12"/>
-      <c r="O30" s="12"/>
-      <c r="P30" s="12"/>
-      <c r="Q30" s="12"/>
-      <c r="R30" s="12"/>
-      <c r="S30" s="12"/>
-      <c r="T30" s="12"/>
-      <c r="U30" s="12"/>
-      <c r="V30" s="12"/>
-      <c r="W30" s="12"/>
-      <c r="X30" s="12"/>
-      <c r="Y30" s="12"/>
-      <c r="Z30" s="12"/>
+      <c r="G30" s="10"/>
+      <c r="H30" s="10"/>
+      <c r="I30" s="10"/>
+      <c r="J30" s="10"/>
+      <c r="K30" s="10"/>
+      <c r="L30" s="10"/>
+      <c r="M30" s="10"/>
+      <c r="N30" s="10"/>
+      <c r="O30" s="10"/>
+      <c r="P30" s="10"/>
+      <c r="Q30" s="10"/>
+      <c r="R30" s="10"/>
+      <c r="S30" s="10"/>
+      <c r="T30" s="10"/>
+      <c r="U30" s="10"/>
+      <c r="V30" s="10"/>
+      <c r="W30" s="10"/>
+      <c r="X30" s="10"/>
+      <c r="Y30" s="10"/>
+      <c r="Z30" s="10"/>
     </row>
     <row x14ac:dyDescent="0.25" r="31" customHeight="1" ht="18.75">
       <c r="A31" s="11" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B31" s="11" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="C31" s="11" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="D31" s="11" t="s">
-        <v>59</v>
+        <v>72</v>
       </c>
       <c r="E31" s="11" t="s">
-        <v>58</v>
+        <v>31</v>
       </c>
       <c r="F31" s="11" t="s">
-        <v>48</v>
-      </c>
-      <c r="G31" s="12"/>
-      <c r="H31" s="12"/>
-      <c r="I31" s="12"/>
-      <c r="J31" s="12"/>
-      <c r="K31" s="12"/>
-      <c r="L31" s="12"/>
-      <c r="M31" s="12"/>
-      <c r="N31" s="12"/>
-      <c r="O31" s="12"/>
-      <c r="P31" s="12"/>
-      <c r="Q31" s="12"/>
-      <c r="R31" s="12"/>
-      <c r="S31" s="12"/>
-      <c r="T31" s="12"/>
-      <c r="U31" s="12"/>
-      <c r="V31" s="12"/>
-      <c r="W31" s="12"/>
-      <c r="X31" s="12"/>
-      <c r="Y31" s="12"/>
-      <c r="Z31" s="12"/>
+        <v>73</v>
+      </c>
+      <c r="G31" s="10"/>
+      <c r="H31" s="10"/>
+      <c r="I31" s="10"/>
+      <c r="J31" s="10"/>
+      <c r="K31" s="10"/>
+      <c r="L31" s="10"/>
+      <c r="M31" s="10"/>
+      <c r="N31" s="10"/>
+      <c r="O31" s="10"/>
+      <c r="P31" s="10"/>
+      <c r="Q31" s="10"/>
+      <c r="R31" s="10"/>
+      <c r="S31" s="10"/>
+      <c r="T31" s="10"/>
+      <c r="U31" s="10"/>
+      <c r="V31" s="10"/>
+      <c r="W31" s="10"/>
+      <c r="X31" s="10"/>
+      <c r="Y31" s="10"/>
+      <c r="Z31" s="10"/>
     </row>
     <row x14ac:dyDescent="0.25" r="32" customHeight="1" ht="18.75">
       <c r="A32" s="11" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B32" s="11" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="C32" s="11" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="D32" s="11" t="s">
-        <v>61</v>
+        <v>74</v>
       </c>
       <c r="E32" s="11" t="s">
-        <v>58</v>
+        <v>31</v>
       </c>
       <c r="F32" s="11" t="s">
-        <v>50</v>
+        <v>75</v>
       </c>
       <c r="G32" s="12"/>
       <c r="H32" s="12"/>
@@ -2082,103 +2095,103 @@
       <c r="Z32" s="12"/>
     </row>
     <row x14ac:dyDescent="0.25" r="33" customHeight="1" ht="18.75">
-      <c r="A33" s="13" t="s">
-        <v>73</v>
-      </c>
-      <c r="B33" s="13" t="s">
-        <v>7</v>
-      </c>
-      <c r="C33" s="13" t="s">
-        <v>44</v>
-      </c>
-      <c r="D33" s="13" t="s">
-        <v>74</v>
-      </c>
-      <c r="E33" s="13" t="s">
-        <v>10</v>
-      </c>
-      <c r="F33" s="13" t="s">
-        <v>48</v>
-      </c>
-      <c r="G33" s="14"/>
-      <c r="H33" s="14"/>
-      <c r="I33" s="14"/>
-      <c r="J33" s="14"/>
-      <c r="K33" s="14"/>
-      <c r="L33" s="14"/>
-      <c r="M33" s="14"/>
-      <c r="N33" s="14"/>
-      <c r="O33" s="14"/>
-      <c r="P33" s="14"/>
-      <c r="Q33" s="14"/>
-      <c r="R33" s="14"/>
-      <c r="S33" s="14"/>
-      <c r="T33" s="14"/>
-      <c r="U33" s="14"/>
-      <c r="V33" s="14"/>
-      <c r="W33" s="14"/>
-      <c r="X33" s="14"/>
-      <c r="Y33" s="14"/>
-      <c r="Z33" s="14"/>
+      <c r="A33" s="11" t="s">
+        <v>64</v>
+      </c>
+      <c r="B33" s="11" t="s">
+        <v>35</v>
+      </c>
+      <c r="C33" s="11" t="s">
+        <v>36</v>
+      </c>
+      <c r="D33" s="11" t="s">
+        <v>60</v>
+      </c>
+      <c r="E33" s="11" t="s">
+        <v>59</v>
+      </c>
+      <c r="F33" s="11" t="s">
+        <v>51</v>
+      </c>
+      <c r="G33" s="12"/>
+      <c r="H33" s="12"/>
+      <c r="I33" s="12"/>
+      <c r="J33" s="12"/>
+      <c r="K33" s="12"/>
+      <c r="L33" s="12"/>
+      <c r="M33" s="12"/>
+      <c r="N33" s="12"/>
+      <c r="O33" s="12"/>
+      <c r="P33" s="12"/>
+      <c r="Q33" s="12"/>
+      <c r="R33" s="12"/>
+      <c r="S33" s="12"/>
+      <c r="T33" s="12"/>
+      <c r="U33" s="12"/>
+      <c r="V33" s="12"/>
+      <c r="W33" s="12"/>
+      <c r="X33" s="12"/>
+      <c r="Y33" s="12"/>
+      <c r="Z33" s="12"/>
     </row>
     <row x14ac:dyDescent="0.25" r="34" customHeight="1" ht="18.75">
-      <c r="A34" s="13" t="s">
-        <v>73</v>
-      </c>
-      <c r="B34" s="13" t="s">
-        <v>7</v>
-      </c>
-      <c r="C34" s="13" t="s">
-        <v>44</v>
-      </c>
-      <c r="D34" s="13" t="s">
-        <v>75</v>
-      </c>
-      <c r="E34" s="13" t="s">
-        <v>10</v>
-      </c>
-      <c r="F34" s="13" t="s">
-        <v>50</v>
-      </c>
-      <c r="G34" s="14"/>
-      <c r="H34" s="14"/>
-      <c r="I34" s="14"/>
-      <c r="J34" s="14"/>
-      <c r="K34" s="14"/>
-      <c r="L34" s="14"/>
-      <c r="M34" s="14"/>
-      <c r="N34" s="14"/>
-      <c r="O34" s="14"/>
-      <c r="P34" s="14"/>
-      <c r="Q34" s="14"/>
-      <c r="R34" s="14"/>
-      <c r="S34" s="14"/>
-      <c r="T34" s="14"/>
-      <c r="U34" s="14"/>
-      <c r="V34" s="14"/>
-      <c r="W34" s="14"/>
-      <c r="X34" s="14"/>
-      <c r="Y34" s="14"/>
-      <c r="Z34" s="14"/>
+      <c r="A34" s="11" t="s">
+        <v>64</v>
+      </c>
+      <c r="B34" s="11" t="s">
+        <v>35</v>
+      </c>
+      <c r="C34" s="11" t="s">
+        <v>36</v>
+      </c>
+      <c r="D34" s="11" t="s">
+        <v>62</v>
+      </c>
+      <c r="E34" s="11" t="s">
+        <v>59</v>
+      </c>
+      <c r="F34" s="11" t="s">
+        <v>53</v>
+      </c>
+      <c r="G34" s="12"/>
+      <c r="H34" s="12"/>
+      <c r="I34" s="12"/>
+      <c r="J34" s="12"/>
+      <c r="K34" s="12"/>
+      <c r="L34" s="12"/>
+      <c r="M34" s="12"/>
+      <c r="N34" s="12"/>
+      <c r="O34" s="12"/>
+      <c r="P34" s="12"/>
+      <c r="Q34" s="12"/>
+      <c r="R34" s="12"/>
+      <c r="S34" s="12"/>
+      <c r="T34" s="12"/>
+      <c r="U34" s="12"/>
+      <c r="V34" s="12"/>
+      <c r="W34" s="12"/>
+      <c r="X34" s="12"/>
+      <c r="Y34" s="12"/>
+      <c r="Z34" s="12"/>
     </row>
     <row x14ac:dyDescent="0.25" r="35" customHeight="1" ht="18.75">
       <c r="A35" s="13" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="B35" s="13" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="C35" s="13" t="s">
-        <v>12</v>
+        <v>47</v>
       </c>
       <c r="D35" s="13" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="E35" s="13" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="F35" s="13" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="G35" s="14"/>
       <c r="H35" s="14"/>
@@ -2203,22 +2216,22 @@
     </row>
     <row x14ac:dyDescent="0.25" r="36" customHeight="1" ht="18.75">
       <c r="A36" s="13" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="B36" s="13" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="C36" s="13" t="s">
-        <v>12</v>
+        <v>47</v>
       </c>
       <c r="D36" s="13" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="E36" s="13" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="F36" s="13" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="G36" s="14"/>
       <c r="H36" s="14"/>
@@ -2243,22 +2256,22 @@
     </row>
     <row x14ac:dyDescent="0.25" r="37" customHeight="1" ht="18.75">
       <c r="A37" s="13" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="B37" s="13" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="C37" s="13" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="D37" s="13" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="E37" s="13" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="F37" s="13" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="G37" s="14"/>
       <c r="H37" s="14"/>
@@ -2283,22 +2296,22 @@
     </row>
     <row x14ac:dyDescent="0.25" r="38" customHeight="1" ht="18.75">
       <c r="A38" s="13" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="B38" s="13" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="C38" s="13" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="D38" s="13" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="E38" s="13" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="F38" s="13" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="G38" s="14"/>
       <c r="H38" s="14"/>
@@ -2323,20 +2336,22 @@
     </row>
     <row x14ac:dyDescent="0.25" r="39" customHeight="1" ht="18.75">
       <c r="A39" s="13" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="B39" s="13" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="C39" s="13" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="D39" s="13" t="s">
-        <v>80</v>
-      </c>
-      <c r="E39" s="13"/>
+        <v>81</v>
+      </c>
+      <c r="E39" s="13" t="s">
+        <v>18</v>
+      </c>
       <c r="F39" s="13" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="G39" s="14"/>
       <c r="H39" s="14"/>
@@ -2361,20 +2376,22 @@
     </row>
     <row x14ac:dyDescent="0.25" r="40" customHeight="1" ht="18.75">
       <c r="A40" s="13" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="B40" s="13" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="C40" s="13" t="s">
-        <v>20</v>
-      </c>
-      <c r="D40" s="14" t="s">
-        <v>81</v>
-      </c>
-      <c r="E40" s="13"/>
+        <v>16</v>
+      </c>
+      <c r="D40" s="13" t="s">
+        <v>82</v>
+      </c>
+      <c r="E40" s="13" t="s">
+        <v>18</v>
+      </c>
       <c r="F40" s="13" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="G40" s="14"/>
       <c r="H40" s="14"/>
@@ -2399,20 +2416,22 @@
     </row>
     <row x14ac:dyDescent="0.25" r="41" customHeight="1" ht="18.75">
       <c r="A41" s="13" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="B41" s="13" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="C41" s="13" t="s">
-        <v>82</v>
+        <v>20</v>
       </c>
       <c r="D41" s="13" t="s">
         <v>83</v>
       </c>
-      <c r="E41" s="13"/>
+      <c r="E41" s="13" t="s">
+        <v>22</v>
+      </c>
       <c r="F41" s="13" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="G41" s="14"/>
       <c r="H41" s="14"/>
@@ -2437,20 +2456,22 @@
     </row>
     <row x14ac:dyDescent="0.25" r="42" customHeight="1" ht="18.75">
       <c r="A42" s="13" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="B42" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="C42" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="D42" s="14" t="s">
+        <v>84</v>
+      </c>
+      <c r="E42" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="C42" s="13" t="s">
-        <v>82</v>
-      </c>
-      <c r="D42" s="13" t="s">
-        <v>84</v>
-      </c>
-      <c r="E42" s="13"/>
       <c r="F42" s="13" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="G42" s="14"/>
       <c r="H42" s="14"/>
@@ -2475,22 +2496,22 @@
     </row>
     <row x14ac:dyDescent="0.25" r="43" customHeight="1" ht="18.75">
       <c r="A43" s="13" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="B43" s="13" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="C43" s="13" t="s">
-        <v>55</v>
+        <v>85</v>
       </c>
       <c r="D43" s="13" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="E43" s="13" t="s">
-        <v>30</v>
+        <v>22</v>
       </c>
       <c r="F43" s="13" t="s">
-        <v>86</v>
+        <v>51</v>
       </c>
       <c r="G43" s="14"/>
       <c r="H43" s="14"/>
@@ -2515,20 +2536,22 @@
     </row>
     <row x14ac:dyDescent="0.25" r="44" customHeight="1" ht="18.75">
       <c r="A44" s="13" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="B44" s="13" t="s">
+        <v>23</v>
+      </c>
+      <c r="C44" s="13" t="s">
+        <v>85</v>
+      </c>
+      <c r="D44" s="13" t="s">
         <v>87</v>
       </c>
-      <c r="C44" s="13" t="s">
-        <v>82</v>
-      </c>
-      <c r="D44" s="13" t="s">
-        <v>83</v>
-      </c>
-      <c r="E44" s="13"/>
+      <c r="E44" s="13" t="s">
+        <v>22</v>
+      </c>
       <c r="F44" s="13" t="s">
-        <v>48</v>
+        <v>53</v>
       </c>
       <c r="G44" s="14"/>
       <c r="H44" s="14"/>
@@ -2553,20 +2576,22 @@
     </row>
     <row x14ac:dyDescent="0.25" r="45" customHeight="1" ht="18.75">
       <c r="A45" s="13" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="B45" s="13" t="s">
-        <v>87</v>
+        <v>28</v>
       </c>
       <c r="C45" s="13" t="s">
-        <v>82</v>
+        <v>29</v>
       </c>
       <c r="D45" s="13" t="s">
         <v>88</v>
       </c>
-      <c r="E45" s="13"/>
+      <c r="E45" s="13" t="s">
+        <v>31</v>
+      </c>
       <c r="F45" s="13" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="G45" s="14"/>
       <c r="H45" s="14"/>
@@ -2591,22 +2616,22 @@
     </row>
     <row x14ac:dyDescent="0.25" r="46" customHeight="1" ht="18.75">
       <c r="A46" s="13" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="B46" s="13" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="C46" s="13" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="D46" s="13" t="s">
         <v>89</v>
       </c>
       <c r="E46" s="13" t="s">
-        <v>90</v>
+        <v>31</v>
       </c>
       <c r="F46" s="13" t="s">
-        <v>48</v>
+        <v>53</v>
       </c>
       <c r="G46" s="14"/>
       <c r="H46" s="14"/>
@@ -2631,22 +2656,22 @@
     </row>
     <row x14ac:dyDescent="0.25" r="47" customHeight="1" ht="18.75">
       <c r="A47" s="13" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="B47" s="13" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C47" s="13" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="D47" s="13" t="s">
+        <v>90</v>
+      </c>
+      <c r="E47" s="13" t="s">
         <v>91</v>
       </c>
-      <c r="E47" s="13" t="s">
-        <v>90</v>
-      </c>
       <c r="F47" s="13" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="G47" s="14"/>
       <c r="H47" s="14"/>
@@ -2671,22 +2696,22 @@
     </row>
     <row x14ac:dyDescent="0.25" r="48" customHeight="1" ht="18.75">
       <c r="A48" s="13" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="B48" s="13" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C48" s="13" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="D48" s="13" t="s">
         <v>92</v>
       </c>
       <c r="E48" s="13" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="F48" s="13" t="s">
-        <v>93</v>
+        <v>53</v>
       </c>
       <c r="G48" s="14"/>
       <c r="H48" s="14"/>
@@ -2709,55 +2734,55 @@
       <c r="Y48" s="14"/>
       <c r="Z48" s="14"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="49" customHeight="1" ht="18.75" customFormat="1" s="15">
-      <c r="A49" s="16" t="s">
+    <row x14ac:dyDescent="0.25" r="49" customHeight="1" ht="18.75">
+      <c r="A49" s="13" t="s">
+        <v>76</v>
+      </c>
+      <c r="B49" s="13" t="s">
+        <v>35</v>
+      </c>
+      <c r="C49" s="13" t="s">
+        <v>36</v>
+      </c>
+      <c r="D49" s="13" t="s">
+        <v>93</v>
+      </c>
+      <c r="E49" s="13" t="s">
+        <v>91</v>
+      </c>
+      <c r="F49" s="13" t="s">
         <v>94</v>
       </c>
-      <c r="B49" s="16" t="s">
-        <v>7</v>
-      </c>
-      <c r="C49" s="16" t="s">
-        <v>44</v>
-      </c>
-      <c r="D49" s="16" t="s">
-        <v>95</v>
-      </c>
-      <c r="E49" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="F49" s="16" t="s">
-        <v>48</v>
-      </c>
-      <c r="G49" s="17"/>
-      <c r="H49" s="17"/>
-      <c r="I49" s="17"/>
-      <c r="J49" s="17"/>
-      <c r="K49" s="17"/>
-      <c r="L49" s="17"/>
-      <c r="M49" s="17"/>
-      <c r="N49" s="17"/>
-      <c r="O49" s="17"/>
-      <c r="P49" s="17"/>
-      <c r="Q49" s="17"/>
-      <c r="R49" s="17"/>
-      <c r="S49" s="17"/>
-      <c r="T49" s="17"/>
-      <c r="U49" s="17"/>
-      <c r="V49" s="17"/>
-      <c r="W49" s="17"/>
-      <c r="X49" s="17"/>
-      <c r="Y49" s="17"/>
-      <c r="Z49" s="17"/>
+      <c r="G49" s="14"/>
+      <c r="H49" s="14"/>
+      <c r="I49" s="14"/>
+      <c r="J49" s="14"/>
+      <c r="K49" s="14"/>
+      <c r="L49" s="14"/>
+      <c r="M49" s="14"/>
+      <c r="N49" s="14"/>
+      <c r="O49" s="14"/>
+      <c r="P49" s="14"/>
+      <c r="Q49" s="14"/>
+      <c r="R49" s="14"/>
+      <c r="S49" s="14"/>
+      <c r="T49" s="14"/>
+      <c r="U49" s="14"/>
+      <c r="V49" s="14"/>
+      <c r="W49" s="14"/>
+      <c r="X49" s="14"/>
+      <c r="Y49" s="14"/>
+      <c r="Z49" s="14"/>
     </row>
     <row x14ac:dyDescent="0.25" r="50" customHeight="1" ht="18.75" customFormat="1" s="15">
       <c r="A50" s="16" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B50" s="16" t="s">
         <v>7</v>
       </c>
       <c r="C50" s="16" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="D50" s="16" t="s">
         <v>96</v>
@@ -2766,7 +2791,7 @@
         <v>10</v>
       </c>
       <c r="F50" s="16" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="G50" s="17"/>
       <c r="H50" s="17"/>
@@ -2791,22 +2816,22 @@
     </row>
     <row x14ac:dyDescent="0.25" r="51" customHeight="1" ht="18.75" customFormat="1" s="15">
       <c r="A51" s="16" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B51" s="16" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="C51" s="16" t="s">
-        <v>12</v>
+        <v>47</v>
       </c>
       <c r="D51" s="16" t="s">
         <v>97</v>
       </c>
       <c r="E51" s="16" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="F51" s="16" t="s">
-        <v>48</v>
+        <v>53</v>
       </c>
       <c r="G51" s="17"/>
       <c r="H51" s="17"/>
@@ -2831,7 +2856,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="52" customHeight="1" ht="18.75" customFormat="1" s="15">
       <c r="A52" s="16" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B52" s="16" t="s">
         <v>11</v>
@@ -2846,7 +2871,7 @@
         <v>14</v>
       </c>
       <c r="F52" s="16" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="G52" s="17"/>
       <c r="H52" s="17"/>
@@ -2871,22 +2896,22 @@
     </row>
     <row x14ac:dyDescent="0.25" r="53" customHeight="1" ht="18.75" customFormat="1" s="15">
       <c r="A53" s="16" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B53" s="16" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="C53" s="16" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="D53" s="16" t="s">
         <v>99</v>
       </c>
       <c r="E53" s="16" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="F53" s="16" t="s">
-        <v>48</v>
+        <v>53</v>
       </c>
       <c r="G53" s="17"/>
       <c r="H53" s="17"/>
@@ -2911,7 +2936,7 @@
     </row>
     <row x14ac:dyDescent="0.25" r="54" customHeight="1" ht="18.75" customFormat="1" s="15">
       <c r="A54" s="16" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B54" s="16" t="s">
         <v>15</v>
@@ -2926,7 +2951,7 @@
         <v>18</v>
       </c>
       <c r="F54" s="16" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="G54" s="17"/>
       <c r="H54" s="17"/>
@@ -2951,17 +2976,23 @@
     </row>
     <row x14ac:dyDescent="0.25" r="55" customHeight="1" ht="18.75" customFormat="1" s="15">
       <c r="A55" s="16" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B55" s="16" t="s">
-        <v>19</v>
-      </c>
-      <c r="C55" s="16"/>
+        <v>15</v>
+      </c>
+      <c r="C55" s="16" t="s">
+        <v>16</v>
+      </c>
       <c r="D55" s="16" t="s">
         <v>101</v>
       </c>
-      <c r="E55" s="16"/>
-      <c r="F55" s="16"/>
+      <c r="E55" s="16" t="s">
+        <v>18</v>
+      </c>
+      <c r="F55" s="16" t="s">
+        <v>53</v>
+      </c>
       <c r="G55" s="17"/>
       <c r="H55" s="17"/>
       <c r="I55" s="17"/>
@@ -2985,14 +3016,20 @@
     </row>
     <row x14ac:dyDescent="0.25" r="56" customHeight="1" ht="18.75" customFormat="1" s="15">
       <c r="A56" s="16" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B56" s="16" t="s">
+        <v>19</v>
+      </c>
+      <c r="C56" s="16" t="s">
+        <v>20</v>
+      </c>
+      <c r="D56" s="16" t="s">
+        <v>102</v>
+      </c>
+      <c r="E56" s="16" t="s">
         <v>22</v>
       </c>
-      <c r="C56" s="16"/>
-      <c r="D56" s="16"/>
-      <c r="E56" s="16"/>
       <c r="F56" s="16"/>
       <c r="G56" s="17"/>
       <c r="H56" s="17"/>
@@ -3017,23 +3054,21 @@
     </row>
     <row x14ac:dyDescent="0.25" r="57" customHeight="1" ht="18.75" customFormat="1" s="15">
       <c r="A57" s="16" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B57" s="16" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="C57" s="16" t="s">
-        <v>55</v>
+        <v>24</v>
       </c>
       <c r="D57" s="16" t="s">
-        <v>102</v>
+        <v>22</v>
       </c>
       <c r="E57" s="16" t="s">
-        <v>30</v>
-      </c>
-      <c r="F57" s="16" t="s">
-        <v>103</v>
-      </c>
+        <v>22</v>
+      </c>
+      <c r="F57" s="16"/>
       <c r="G57" s="17"/>
       <c r="H57" s="17"/>
       <c r="I57" s="17"/>
@@ -3057,22 +3092,22 @@
     </row>
     <row x14ac:dyDescent="0.25" r="58" customHeight="1" ht="18.75" customFormat="1" s="15">
       <c r="A58" s="16" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B58" s="16" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="C58" s="16" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="D58" s="16" t="s">
+        <v>103</v>
+      </c>
+      <c r="E58" s="16" t="s">
+        <v>31</v>
+      </c>
+      <c r="F58" s="16" t="s">
         <v>104</v>
-      </c>
-      <c r="E58" s="16" t="s">
-        <v>90</v>
-      </c>
-      <c r="F58" s="16" t="s">
-        <v>48</v>
       </c>
       <c r="G58" s="17"/>
       <c r="H58" s="17"/>
@@ -3097,22 +3132,22 @@
     </row>
     <row x14ac:dyDescent="0.25" r="59" customHeight="1" ht="18.75" customFormat="1" s="15">
       <c r="A59" s="16" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B59" s="16" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C59" s="16" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="D59" s="16" t="s">
         <v>105</v>
       </c>
       <c r="E59" s="16" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="F59" s="16" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="G59" s="17"/>
       <c r="H59" s="17"/>
@@ -3136,12 +3171,24 @@
       <c r="Z59" s="17"/>
     </row>
     <row x14ac:dyDescent="0.25" r="60" customHeight="1" ht="18.75" customFormat="1" s="15">
-      <c r="A60" s="16"/>
-      <c r="B60" s="16"/>
-      <c r="C60" s="16"/>
-      <c r="D60" s="16"/>
-      <c r="E60" s="16"/>
-      <c r="F60" s="16"/>
+      <c r="A60" s="16" t="s">
+        <v>95</v>
+      </c>
+      <c r="B60" s="16" t="s">
+        <v>35</v>
+      </c>
+      <c r="C60" s="16" t="s">
+        <v>36</v>
+      </c>
+      <c r="D60" s="16" t="s">
+        <v>106</v>
+      </c>
+      <c r="E60" s="16" t="s">
+        <v>91</v>
+      </c>
+      <c r="F60" s="16" t="s">
+        <v>53</v>
+      </c>
       <c r="G60" s="17"/>
       <c r="H60" s="17"/>
       <c r="I60" s="17"/>
@@ -30379,6 +30426,34 @@
       <c r="Y1032" s="17"/>
       <c r="Z1032" s="17"/>
     </row>
+    <row x14ac:dyDescent="0.25" r="1033" customHeight="1" ht="18.75" customFormat="1" s="15">
+      <c r="A1033" s="16"/>
+      <c r="B1033" s="16"/>
+      <c r="C1033" s="16"/>
+      <c r="D1033" s="16"/>
+      <c r="E1033" s="16"/>
+      <c r="F1033" s="16"/>
+      <c r="G1033" s="17"/>
+      <c r="H1033" s="17"/>
+      <c r="I1033" s="17"/>
+      <c r="J1033" s="17"/>
+      <c r="K1033" s="17"/>
+      <c r="L1033" s="17"/>
+      <c r="M1033" s="17"/>
+      <c r="N1033" s="17"/>
+      <c r="O1033" s="17"/>
+      <c r="P1033" s="17"/>
+      <c r="Q1033" s="17"/>
+      <c r="R1033" s="17"/>
+      <c r="S1033" s="17"/>
+      <c r="T1033" s="17"/>
+      <c r="U1033" s="17"/>
+      <c r="V1033" s="17"/>
+      <c r="W1033" s="17"/>
+      <c r="X1033" s="17"/>
+      <c r="Y1033" s="17"/>
+      <c r="Z1033" s="17"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>